<commit_message>
Update impact ball description and terrain points
</commit_message>
<xml_diff>
--- a/LubanConfig/DataTables/Datas/#TerrainParam.xlsx
+++ b/LubanConfig/DataTables/Datas/#TerrainParam.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Github\monster-ball\LubanConfig\DataTables\Datas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72ADC82A-E0A3-49AB-9EC5-6E3B69D4E5E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE19FA4-2612-4B7A-A82B-951E0E45FCAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1812" yWindow="1812" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TerrainParam " sheetId="1" r:id="rId1"/>
@@ -639,10 +639,10 @@
     <row r="5" spans="1:28" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" s="1">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="C5" s="1">
-        <v>500</v>
+        <v>75</v>
       </c>
       <c r="D5" s="1">
         <v>1.25</v>
@@ -651,13 +651,13 @@
         <v>5</v>
       </c>
       <c r="F5" s="1">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="G5" s="1">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="H5" s="1">
-        <v>750</v>
+        <v>250</v>
       </c>
       <c r="I5" s="1">
         <v>1000</v>

</xml_diff>